<commit_message>
Percentile tables and MCDI calculations
</commit_message>
<xml_diff>
--- a/public/templates/EPICS project-Variable needed-Output.xlsx
+++ b/public/templates/EPICS project-Variable needed-Output.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cometmail-my.sharepoint.com/personal/jxx240004_utdallas_edu/Documents/MCDI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="316" documentId="8_{8BB48137-E22C-4444-A280-13E234375999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C0C62E0-A184-4680-9CE6-06950D60A56A}"/>
+  <xr:revisionPtr revIDLastSave="322" documentId="8_{8BB48137-E22C-4444-A280-13E234375999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC5E49EE-391D-4820-8178-1E4C3479034F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{DF9DA3B6-2788-4AF3-83F2-DBC0B5DFFB5F}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{DF9DA3B6-2788-4AF3-83F2-DBC0B5DFFB5F}"/>
   </bookViews>
   <sheets>
     <sheet name="colorkey" sheetId="12" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="78">
   <si>
     <t>chname_reg</t>
   </si>
@@ -88,12 +88,6 @@
     <t>total_expressive_span</t>
   </si>
   <si>
-    <t>total_receptive=total_receptive_span + total_receptive_eng</t>
-  </si>
-  <si>
-    <t>total_expressive=total_expressive_span + total_expressive_eng</t>
-  </si>
-  <si>
     <t>es2_english_total</t>
   </si>
   <si>
@@ -275,6 +269,15 @@
   </si>
   <si>
     <t>mcdimandarin_timestamp</t>
+  </si>
+  <si>
+    <t>total_receptive</t>
+  </si>
+  <si>
+    <t>total_expressive</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> for percentile calculation</t>
   </si>
 </sst>
 </file>
@@ -369,7 +372,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -385,12 +388,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.749992370372631"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -457,7 +454,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -478,9 +475,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -500,9 +494,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -904,53 +895,53 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:1" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+    <row r="4" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+    <row r="7" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+    <row r="11" spans="1:1" ht="26.25" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+    <row r="12" spans="1:1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="26.25" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
     <row r="13" spans="1:1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
-        <v>71</v>
+      <c r="A13" s="13" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -970,10 +961,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="2" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -991,14 +982,14 @@
       <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>56</v>
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>54</v>
       </c>
       <c r="K1" s="5" t="s">
         <v>5</v>
@@ -1006,54 +997,54 @@
       <c r="L1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="O1" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="P1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="O1" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="P1" s="17" t="s">
-        <v>44</v>
-      </c>
       <c r="Q1" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E3" s="16">
+        <v>45698</v>
+      </c>
+      <c r="F3" t="s">
         <v>46</v>
-      </c>
-      <c r="D3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="18">
-        <v>45698</v>
-      </c>
-      <c r="F3" t="s">
-        <v>48</v>
       </c>
       <c r="G3">
         <v>11</v>
@@ -1074,30 +1065,30 @@
         <v>30</v>
       </c>
       <c r="O3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="P3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="16">
+        <v>45677</v>
+      </c>
+      <c r="F4" t="s">
         <v>50</v>
-      </c>
-      <c r="D4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="18">
-        <v>45677</v>
-      </c>
-      <c r="F4" t="s">
-        <v>52</v>
       </c>
       <c r="G4">
         <v>12</v>
@@ -1112,16 +1103,16 @@
         <v>0</v>
       </c>
       <c r="M4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="N4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="O4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="P4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1141,10 +1132,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -1162,75 +1153,75 @@
       <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>56</v>
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>54</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="L1" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="M1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="17" t="s">
-        <v>44</v>
-      </c>
       <c r="N1" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E3" s="19">
+      <c r="E3" s="17">
         <v>45279</v>
       </c>
-      <c r="F3" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="20">
+      <c r="F3" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="18">
         <v>22</v>
       </c>
       <c r="H3">
         <v>20</v>
       </c>
-      <c r="I3" s="20">
+      <c r="I3" s="18">
         <v>2</v>
       </c>
-      <c r="K3" s="20">
+      <c r="K3" s="18">
         <v>26</v>
       </c>
       <c r="L3">
         <v>29</v>
       </c>
       <c r="M3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1250,10 +1241,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" s="6" customFormat="1" ht="141.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -1271,14 +1262,14 @@
       <c r="G1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>56</v>
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>54</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>10</v>
@@ -1292,164 +1283,164 @@
       <c r="N1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="16" t="s">
+      <c r="O1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q1" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="R1" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="S1" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="T1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="S1" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="T1" s="17" t="s">
-        <v>44</v>
-      </c>
       <c r="U1" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="O2" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="P2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="26">
+        <v>49</v>
+      </c>
+      <c r="E3" s="24">
         <v>45534</v>
       </c>
-      <c r="F3" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="27">
+      <c r="F3" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="25">
         <v>13</v>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="25">
         <v>13</v>
       </c>
-      <c r="I3" s="28">
-        <v>1</v>
-      </c>
-      <c r="J3" s="28">
-        <v>1</v>
-      </c>
-      <c r="K3" s="20">
+      <c r="I3" s="26">
+        <v>1</v>
+      </c>
+      <c r="J3" s="26">
+        <v>1</v>
+      </c>
+      <c r="K3" s="18">
         <v>18</v>
       </c>
-      <c r="L3" s="27">
+      <c r="L3" s="25">
         <v>6</v>
       </c>
-      <c r="M3" s="27">
+      <c r="M3" s="25">
         <v>16</v>
       </c>
-      <c r="N3" s="27">
+      <c r="N3" s="25">
         <v>3</v>
       </c>
-      <c r="O3" s="29">
+      <c r="O3" s="27">
         <v>34</v>
       </c>
-      <c r="P3" s="29">
+      <c r="P3" s="27">
         <v>9</v>
       </c>
-      <c r="Q3" s="29">
+      <c r="Q3" s="27">
         <v>58.75</v>
       </c>
-      <c r="R3" s="29">
+      <c r="R3" s="27">
         <v>70</v>
       </c>
       <c r="S3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="T3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="26">
+        <v>49</v>
+      </c>
+      <c r="E4" s="24">
         <v>45604</v>
       </c>
-      <c r="F4" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="G4" s="27">
+      <c r="F4" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="25">
         <v>11</v>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="25">
         <v>11</v>
       </c>
-      <c r="I4" s="28">
-        <v>1</v>
-      </c>
-      <c r="J4" s="28">
-        <v>1</v>
-      </c>
-      <c r="K4" s="20">
+      <c r="I4" s="26">
+        <v>1</v>
+      </c>
+      <c r="J4" s="26">
+        <v>1</v>
+      </c>
+      <c r="K4" s="18">
         <v>3</v>
       </c>
-      <c r="L4" s="27">
+      <c r="L4" s="25">
         <v>0</v>
       </c>
-      <c r="M4" s="27">
+      <c r="M4" s="25">
         <v>5</v>
       </c>
-      <c r="N4" s="27">
-        <v>1</v>
-      </c>
-      <c r="O4" s="29">
+      <c r="N4" s="25">
+        <v>1</v>
+      </c>
+      <c r="O4" s="27">
         <v>8</v>
       </c>
-      <c r="P4" s="29">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="29">
+      <c r="P4" s="27">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="27">
         <v>39</v>
       </c>
-      <c r="R4" s="29">
+      <c r="R4" s="27">
         <v>40</v>
       </c>
       <c r="S4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="T4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1466,10 +1457,10 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:16" ht="141.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -1487,184 +1478,184 @@
       <c r="G1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N1" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="N1" s="16" t="s">
+      <c r="O1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="O1" s="17" t="s">
-        <v>44</v>
-      </c>
       <c r="P1" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" t="s">
-        <v>46</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="E3" s="28">
+        <v>45299</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="18">
+        <v>21</v>
+      </c>
+      <c r="H3" s="18">
+        <v>21</v>
+      </c>
+      <c r="I3" s="29">
+        <v>1</v>
+      </c>
+      <c r="J3" s="29">
+        <v>1</v>
+      </c>
+      <c r="K3" s="18">
+        <v>3</v>
+      </c>
+      <c r="L3" s="18">
+        <v>21</v>
+      </c>
+      <c r="M3" s="18">
+        <v>24</v>
+      </c>
+      <c r="N3" s="19">
+        <v>31.67</v>
+      </c>
+      <c r="O3" t="s">
         <v>47</v>
-      </c>
-      <c r="E3" s="30">
-        <v>45299</v>
-      </c>
-      <c r="F3" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="G3" s="20">
-        <v>21</v>
-      </c>
-      <c r="H3" s="20">
-        <v>21</v>
-      </c>
-      <c r="I3" s="31">
-        <v>1</v>
-      </c>
-      <c r="J3" s="31">
-        <v>1</v>
-      </c>
-      <c r="K3" s="20">
-        <v>3</v>
-      </c>
-      <c r="L3" s="20">
-        <v>21</v>
-      </c>
-      <c r="M3" s="20">
-        <v>24</v>
-      </c>
-      <c r="N3" s="21">
-        <v>31.67</v>
-      </c>
-      <c r="O3" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="30">
+        <v>49</v>
+      </c>
+      <c r="E4" s="28">
         <v>45149</v>
       </c>
-      <c r="F4" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="G4" s="20">
+      <c r="F4" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="18">
         <v>26</v>
       </c>
-      <c r="H4" s="20">
+      <c r="H4" s="18">
         <v>26</v>
       </c>
-      <c r="I4" s="31">
-        <v>1</v>
-      </c>
-      <c r="J4" s="31">
-        <v>1</v>
-      </c>
-      <c r="K4" s="20">
+      <c r="I4" s="29">
+        <v>1</v>
+      </c>
+      <c r="J4" s="29">
+        <v>1</v>
+      </c>
+      <c r="K4" s="18">
         <v>0</v>
       </c>
-      <c r="L4" s="20">
+      <c r="L4" s="18">
         <v>13</v>
       </c>
-      <c r="M4" s="20">
+      <c r="M4" s="18">
         <v>13</v>
       </c>
-      <c r="N4" s="21">
+      <c r="N4" s="19">
         <v>6.67</v>
       </c>
       <c r="O4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="28">
+        <v>45099</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" s="18">
+        <v>28</v>
+      </c>
+      <c r="H5" s="18">
+        <v>28</v>
+      </c>
+      <c r="I5" s="29">
+        <v>1</v>
+      </c>
+      <c r="J5" s="29">
+        <v>1</v>
+      </c>
+      <c r="K5" s="18">
+        <v>2</v>
+      </c>
+      <c r="L5" s="18">
+        <v>5</v>
+      </c>
+      <c r="M5" s="18">
+        <v>7</v>
+      </c>
+      <c r="N5" t="s">
         <v>51</v>
       </c>
-      <c r="E5" s="30">
-        <v>45099</v>
-      </c>
-      <c r="F5" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="G5" s="20">
-        <v>28</v>
-      </c>
-      <c r="H5" s="20">
-        <v>28</v>
-      </c>
-      <c r="I5" s="31">
-        <v>1</v>
-      </c>
-      <c r="J5" s="31">
-        <v>1</v>
-      </c>
-      <c r="K5" s="20">
-        <v>2</v>
-      </c>
-      <c r="L5" s="20">
-        <v>5</v>
-      </c>
-      <c r="M5" s="20">
-        <v>7</v>
-      </c>
-      <c r="N5" t="s">
-        <v>53</v>
-      </c>
       <c r="O5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1681,10 +1672,10 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:21" s="3" customFormat="1" ht="141.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -1702,185 +1693,185 @@
       <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q1" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="R1" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="M1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" s="16" t="s">
+      <c r="S1" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="R1" s="16" t="s">
+      <c r="T1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="S1" s="17" t="s">
-        <v>43</v>
-      </c>
-      <c r="T1" s="17" t="s">
-        <v>44</v>
-      </c>
       <c r="U1" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" t="s">
+        <v>21</v>
+      </c>
+      <c r="O2" t="s">
+        <v>22</v>
+      </c>
+      <c r="P2" t="s">
         <v>23</v>
-      </c>
-      <c r="H2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O2" t="s">
-        <v>24</v>
-      </c>
-      <c r="P2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="26">
+        <v>67</v>
+      </c>
+      <c r="E3" s="24">
         <v>45534</v>
       </c>
-      <c r="F3" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="27">
+      <c r="F3" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="25">
         <v>13</v>
       </c>
-      <c r="H3" s="27">
+      <c r="H3" s="25">
         <v>13</v>
       </c>
-      <c r="I3" s="28">
-        <v>1</v>
-      </c>
-      <c r="J3" s="28">
+      <c r="I3" s="26">
+        <v>1</v>
+      </c>
+      <c r="J3" s="26">
         <v>2</v>
       </c>
-      <c r="K3" s="28">
+      <c r="K3" s="26">
         <v>34</v>
       </c>
-      <c r="L3" s="28">
+      <c r="L3" s="26">
         <v>2</v>
       </c>
-      <c r="M3" s="28">
+      <c r="M3" s="26">
         <v>200</v>
       </c>
-      <c r="N3" s="28">
+      <c r="N3" s="26">
         <v>1</v>
       </c>
       <c r="O3">
         <v>234</v>
       </c>
-      <c r="P3" s="32">
+      <c r="P3" s="30">
         <v>3</v>
       </c>
-      <c r="Q3" s="32">
+      <c r="Q3" s="30">
         <v>80</v>
       </c>
-      <c r="R3" s="32">
+      <c r="R3" s="30">
         <v>60</v>
       </c>
       <c r="S3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="T3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="24">
+        <v>45604</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>50</v>
       </c>
-      <c r="D4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E4" s="26">
-        <v>45604</v>
-      </c>
-      <c r="F4" s="27" t="s">
-        <v>52</v>
-      </c>
-      <c r="G4" s="27">
+      <c r="G4" s="25">
         <v>11</v>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="25">
         <v>11</v>
       </c>
-      <c r="I4" s="28">
-        <v>1</v>
-      </c>
-      <c r="J4" s="28">
+      <c r="I4" s="26">
+        <v>1</v>
+      </c>
+      <c r="J4" s="26">
         <v>2</v>
       </c>
-      <c r="K4" s="28">
+      <c r="K4" s="26">
         <v>35</v>
       </c>
-      <c r="L4" s="28">
+      <c r="L4" s="26">
         <v>3</v>
       </c>
-      <c r="M4" s="28">
+      <c r="M4" s="26">
         <v>520</v>
       </c>
-      <c r="N4" s="28">
+      <c r="N4" s="26">
         <v>1</v>
       </c>
       <c r="O4">
         <v>555</v>
       </c>
-      <c r="P4" s="32">
+      <c r="P4" s="30">
         <v>4</v>
       </c>
       <c r="Q4" t="s">
-        <v>68</v>
-      </c>
-      <c r="R4" s="32">
+        <v>66</v>
+      </c>
+      <c r="R4" s="30">
         <v>50</v>
       </c>
       <c r="S4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="T4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1897,10 +1888,10 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:16" ht="141.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -1918,68 +1909,68 @@
       <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="L1" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="N1" s="16" t="s">
+      <c r="O1" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="O1" s="17" t="s">
-        <v>44</v>
-      </c>
       <c r="P1" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="F2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="33">
+        <v>67</v>
+      </c>
+      <c r="E3" s="31">
         <v>45084</v>
       </c>
       <c r="F3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G3" s="35">
+        <v>46</v>
+      </c>
+      <c r="G3" s="33">
         <v>28</v>
       </c>
-      <c r="H3" s="35">
+      <c r="H3" s="33">
         <v>28</v>
       </c>
       <c r="I3">
@@ -1988,10 +1979,10 @@
       <c r="J3">
         <v>2</v>
       </c>
-      <c r="K3" s="36">
+      <c r="K3" s="34">
         <v>150</v>
       </c>
-      <c r="L3" s="35">
+      <c r="L3" s="33">
         <v>451</v>
       </c>
       <c r="M3">
@@ -2001,32 +1992,32 @@
         <v>80.06</v>
       </c>
       <c r="O3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>69</v>
-      </c>
-      <c r="E4" s="34">
+        <v>67</v>
+      </c>
+      <c r="E4" s="32">
         <v>45294</v>
       </c>
       <c r="F4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G4" s="35">
+        <v>50</v>
+      </c>
+      <c r="G4" s="33">
         <v>21</v>
       </c>
-      <c r="H4" s="35">
+      <c r="H4" s="33">
         <v>21</v>
       </c>
       <c r="I4">
@@ -2035,10 +2026,10 @@
       <c r="J4">
         <v>2</v>
       </c>
-      <c r="K4" s="36">
+      <c r="K4" s="34">
         <v>37</v>
       </c>
-      <c r="L4" s="35">
+      <c r="L4" s="33">
         <v>146</v>
       </c>
       <c r="M4">
@@ -2048,7 +2039,7 @@
         <v>50.05</v>
       </c>
       <c r="O4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -2068,10 +2059,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="2" customFormat="1" ht="99.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
@@ -2089,17 +2080,17 @@
       <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="K1" s="12" t="s">
-        <v>59</v>
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>57</v>
       </c>
       <c r="L1" s="5" t="s">
         <v>5</v>
@@ -2108,137 +2099,137 @@
         <v>6</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" t="s">
         <v>62</v>
       </c>
-      <c r="B3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E3" s="19">
+      <c r="E3" s="17">
         <v>45524</v>
       </c>
       <c r="F3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="20">
+        <v>50</v>
+      </c>
+      <c r="G3" s="18">
         <v>14</v>
       </c>
       <c r="H3">
         <v>14</v>
       </c>
-      <c r="I3" s="20">
-        <v>1</v>
-      </c>
-      <c r="J3" s="20">
+      <c r="I3" s="18">
+        <v>1</v>
+      </c>
+      <c r="J3" s="18">
         <v>3</v>
       </c>
-      <c r="K3" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="L3" s="20">
+      <c r="K3" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="L3" s="18">
         <v>19</v>
       </c>
-      <c r="M3" s="21">
+      <c r="M3" s="19">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
         <v>62</v>
       </c>
-      <c r="B4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C4" t="s">
-        <v>63</v>
-      </c>
-      <c r="D4" t="s">
-        <v>64</v>
-      </c>
-      <c r="E4" s="19">
+      <c r="E4" s="17">
         <v>45478</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G4" s="20">
+        <v>46</v>
+      </c>
+      <c r="G4" s="18">
         <v>15</v>
       </c>
       <c r="H4">
         <v>15</v>
       </c>
-      <c r="I4" s="20">
-        <v>1</v>
-      </c>
-      <c r="J4" s="20">
+      <c r="I4" s="18">
+        <v>1</v>
+      </c>
+      <c r="J4" s="18">
         <v>3</v>
       </c>
-      <c r="K4" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="L4" s="20">
+      <c r="K4" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="L4" s="18">
         <v>28</v>
       </c>
-      <c r="M4" s="21">
+      <c r="M4" s="19">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:15" s="22" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+    <row r="5" spans="1:15" s="20" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D5" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>64</v>
-      </c>
-      <c r="E5" s="23">
+      <c r="E5" s="21">
         <v>45145</v>
       </c>
-      <c r="F5" s="22" t="s">
-        <v>48</v>
-      </c>
-      <c r="G5" s="24">
+      <c r="F5" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="22">
         <v>16</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="20">
         <v>16</v>
       </c>
-      <c r="I5" s="24">
-        <v>1</v>
-      </c>
-      <c r="J5" s="24">
+      <c r="I5" s="22">
+        <v>1</v>
+      </c>
+      <c r="J5" s="22">
         <v>3</v>
       </c>
-      <c r="K5" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="L5" s="25">
+      <c r="K5" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="L5" s="23">
         <v>21</v>
       </c>
-      <c r="M5" s="25">
+      <c r="M5" s="23">
         <v>2</v>
       </c>
     </row>
@@ -2281,17 +2272,17 @@
       <c r="G1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I1" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="J1" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="K1" s="12" t="s">
-        <v>59</v>
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>57</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>6</v>
@@ -2299,82 +2290,82 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="19">
+        <v>49</v>
+      </c>
+      <c r="E3" s="17">
         <v>45347</v>
       </c>
-      <c r="F3" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="20">
+      <c r="F3" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="18">
         <v>20</v>
       </c>
       <c r="H3">
         <v>20</v>
       </c>
-      <c r="I3" s="20">
-        <v>1</v>
-      </c>
-      <c r="J3" s="20">
+      <c r="I3" s="18">
+        <v>1</v>
+      </c>
+      <c r="J3" s="18">
         <v>3</v>
       </c>
-      <c r="K3" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="L3" s="21">
+      <c r="K3" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="L3" s="19">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" s="19">
+        <v>49</v>
+      </c>
+      <c r="E4" s="17">
         <v>45233</v>
       </c>
-      <c r="F4" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="G4" s="20">
+      <c r="F4" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="18">
         <v>23</v>
       </c>
       <c r="H4">
         <v>23</v>
       </c>
-      <c r="I4" s="20">
-        <v>1</v>
-      </c>
-      <c r="J4" s="20">
+      <c r="I4" s="18">
+        <v>1</v>
+      </c>
+      <c r="J4" s="18">
         <v>3</v>
       </c>
-      <c r="K4" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="L4" s="21">
+      <c r="K4" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="L4" s="19">
         <v>34</v>
       </c>
     </row>

</xml_diff>